<commit_message>
Draft private round rankings and flexible quiz flow
</commit_message>
<xml_diff>
--- a/dist/question-bank-template.xlsx
+++ b/dist/question-bank-template.xlsx
@@ -847,10 +847,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H10"/>
-  <dataValidations count="2">
-    <dataValidation sqref="A2:A61" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="請使用下拉選單的值" type="list">
-      <formula1>"1,2,3"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="H2:H61" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="請使用下拉選單的值" type="list">
       <formula1>"A,B,C,D"</formula1>
     </dataValidation>
@@ -888,7 +885,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>依回合 1、2、3 排列，每回合 1～20 題，同一回合名稱一致。</t>
+          <t>依回合正整數順序排列，同一回合名稱一致。</t>
         </is>
       </c>
     </row>

</xml_diff>